<commit_message>
BRD-11 User Access Maintenance screenshots retaken in the BDO style-guide presentation on a fresh seed stack: 93 images; FRS, guide deck, sign-off workbook and UX documents 07 to 09 rebuilt at v2.0 with issue 2.2 change CHG-UA-2.2-01; the second-approval shot taken before walkthrough B, Sessions from the user's row menu, the separation-of-duties row menu in the screen specification and fixes for the data access messages
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-11_User_Access_Maintenance/08_BIBS_UXScreens_BRD-11_User_Access_Maintenance_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-11_User_Access_Maintenance/08_BIBS_UXScreens_BRD-11_User_Access_Maintenance_v2.0.xlsx
@@ -688,7 +688,7 @@
 Mandatory: Yes
 Format: Y or N
 Allowed values: Y or N
-Example: N</t>
+Example: Y</t>
       </text>
     </comment>
     <comment ref="O16" authorId="0" shapeId="0">
@@ -697,7 +697,8 @@
 The change reference (comment, change request or issue change) that changed the image
 Mandatory: Conditional: when Changed in this issue is Y
 Format: Reference
-Allowed values: Free entry</t>
+Allowed values: Free entry
+Example: CHG-UA-2.2-01</t>
       </text>
     </comment>
   </commentList>
@@ -1072,7 +1073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:I37"/>
+  <dimension ref="A2:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1347,7 +1348,7 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>99 screen images of 33 screens; 13 changed in this issue</t>
+          <t>99 screen images of 33 screens; 77 changed in this issue</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
@@ -1519,43 +1520,47 @@
       </c>
       <c r="I30" s="5" t="n"/>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Lists in the BDO style guide: outlined status pills, alternating white and Background Blue rows, a long list scrolling inside its card with the header row in view, names instead of codes, due dates on one line with the overdue icon and ages in words; every image of the set retaken</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>SCR-UA-01, SCR-UA-02, SCR-UA-03, SCR-UA-04, SCR-UA-05, SCR-UA-06, SCR-UA-07, SCR-UA-08, SCR-UA-09, SCR-UA-10, SCR-UA-11, SCR-UA-12, SCR-UA-13, SCR-UA-14, SCR-UA-15, SCR-UA-16, SCR-UA-17, SCR-UA-18, SCR-UA-19</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Other sheets</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Sheet</t>
-        </is>
-      </c>
-      <c r="B33" s="18" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>What it holds</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="5" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Reference lists</t>
         </is>
       </c>
       <c r="B34" s="18" t="n"/>
       <c r="C34" s="5" t="n"/>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>The lists of the drop-downs: states and UXD statuses</t>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>What it holds</t>
         </is>
       </c>
       <c r="E34" s="18" t="n"/>
@@ -1567,14 +1572,14 @@
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Questions and comments</t>
+          <t>Reference lists</t>
         </is>
       </c>
       <c r="B35" s="18" t="n"/>
       <c r="C35" s="5" t="n"/>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>Questions and comments of the UX Design team, with the answer</t>
+          <t>The lists of the drop-downs: states and UXD statuses</t>
         </is>
       </c>
       <c r="E35" s="18" t="n"/>
@@ -1583,8 +1588,27 @@
       <c r="H35" s="18" t="n"/>
       <c r="I35" s="5" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Questions and comments</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>Questions and comments of the UX Design team, with the answer</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="n"/>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Prepared by iorta TechNXT for BDOI. Confidential – BDOI.</t>
         </is>
@@ -1592,7 +1616,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A21:I22"/>
-  <mergeCells count="41">
+  <mergeCells count="44">
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="C30:G30"/>
@@ -1600,23 +1624,23 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C9:H9"/>
     <mergeCell ref="B16:I16"/>
+    <mergeCell ref="H31:I31"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C26:G26"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="C11:H11"/>
     <mergeCell ref="H25:I25"/>
     <mergeCell ref="C29:G29"/>
-    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C25:G25"/>
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="B14:I14"/>
+    <mergeCell ref="C31:G31"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="B17:I17"/>
-    <mergeCell ref="D33:I33"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="C27:G27"/>
     <mergeCell ref="D35:I35"/>
@@ -1626,12 +1650,15 @@
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="D34:I34"/>
     <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="B15:I15"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:G28"/>
+    <mergeCell ref="D36:I36"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A31:B31"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="H26:I26"/>
   </mergeCells>
@@ -1661,8 +1688,8 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="I22" location="'UX screen register'!A1"/>
-    <hyperlink ref="A34" location="'Reference lists'!A1"/>
-    <hyperlink ref="A35" location="'Questions and comments'!A1"/>
+    <hyperlink ref="A35" location="'Reference lists'!A1"/>
+    <hyperlink ref="A36" location="'Questions and comments'!A1"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
@@ -2301,10 +2328,14 @@
       <c r="M17" s="43" t="n"/>
       <c r="N17" s="43" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O17" s="43" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O17" s="43" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="45" t="inlineStr">
@@ -2361,10 +2392,14 @@
       <c r="M18" s="45" t="n"/>
       <c r="N18" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O18" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O18" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="45" t="inlineStr">
@@ -2421,10 +2456,14 @@
       <c r="M19" s="45" t="n"/>
       <c r="N19" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O19" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O19" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="45" t="inlineStr">
@@ -2481,10 +2520,14 @@
       <c r="M20" s="45" t="n"/>
       <c r="N20" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O20" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O20" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="45" t="inlineStr">
@@ -2541,10 +2584,14 @@
       <c r="M21" s="45" t="n"/>
       <c r="N21" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O21" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O21" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="45" t="inlineStr">
@@ -2601,10 +2648,14 @@
       <c r="M22" s="45" t="n"/>
       <c r="N22" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O22" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O22" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="45" t="inlineStr">
@@ -2661,10 +2712,14 @@
       <c r="M23" s="45" t="n"/>
       <c r="N23" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O23" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O23" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="45" t="inlineStr">
@@ -2721,10 +2776,14 @@
       <c r="M24" s="45" t="n"/>
       <c r="N24" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O24" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O24" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="45" t="inlineStr">
@@ -2781,10 +2840,14 @@
       <c r="M25" s="45" t="n"/>
       <c r="N25" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O25" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O25" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="45" t="inlineStr">
@@ -2841,10 +2904,14 @@
       <c r="M26" s="45" t="n"/>
       <c r="N26" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O26" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O26" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="45" t="inlineStr">
@@ -2906,7 +2973,7 @@
       </c>
       <c r="O27" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -2970,7 +3037,7 @@
       </c>
       <c r="O28" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3101,7 @@
       </c>
       <c r="O29" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-05</t>
+          <t>CHG-UA-2.1-05, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3165,7 @@
       </c>
       <c r="O30" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-05</t>
+          <t>CHG-UA-2.1-05, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3229,7 @@
       </c>
       <c r="O31" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-05</t>
+          <t>CHG-UA-2.1-05, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3293,7 @@
       </c>
       <c r="O32" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-05</t>
+          <t>CHG-UA-2.1-05, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3357,7 @@
       </c>
       <c r="O33" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01, CHG-UA-2.1-02, CHG-UA-2.1-03, CHG-UA-2.1-04</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.1-02, CHG-UA-2.1-03, CHG-UA-2.1-04, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3421,7 @@
       </c>
       <c r="O34" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01, CHG-UA-2.1-04</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.1-04, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3485,7 @@
       </c>
       <c r="O35" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01, CHG-UA-2.1-02, CHG-UA-2.1-03, CHG-UA-2.1-04</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.1-02, CHG-UA-2.1-03, CHG-UA-2.1-04, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3549,7 @@
       </c>
       <c r="O36" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01, CHG-UA-2.1-02, CHG-UA-2.1-03, CHG-UA-2.1-04</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.1-02, CHG-UA-2.1-03, CHG-UA-2.1-04, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3613,7 @@
       </c>
       <c r="O37" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-04</t>
+          <t>CHG-UA-2.1-04, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3605,10 +3672,14 @@
       <c r="M38" s="45" t="n"/>
       <c r="N38" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O38" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O38" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="45" t="inlineStr">
@@ -3665,10 +3736,14 @@
       <c r="M39" s="45" t="n"/>
       <c r="N39" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O39" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O39" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="45" t="inlineStr">
@@ -3730,7 +3805,7 @@
       </c>
       <c r="O40" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01, CHG-UA-2.1-02</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.1-02, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3869,7 @@
       </c>
       <c r="O41" s="45" t="inlineStr">
         <is>
-          <t>CHG-UA-2.1-01</t>
+          <t>CHG-UA-2.1-01, CHG-UA-2.2-01</t>
         </is>
       </c>
     </row>
@@ -3853,10 +3928,14 @@
       <c r="M42" s="45" t="n"/>
       <c r="N42" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O42" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O42" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="45" t="inlineStr">
@@ -3913,10 +3992,14 @@
       <c r="M43" s="45" t="n"/>
       <c r="N43" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O43" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O43" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="45" t="inlineStr">
@@ -3973,10 +4056,14 @@
       <c r="M44" s="45" t="n"/>
       <c r="N44" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O44" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O44" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="45" t="inlineStr">
@@ -4033,10 +4120,14 @@
       <c r="M45" s="45" t="n"/>
       <c r="N45" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O45" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O45" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="45" t="inlineStr">
@@ -4093,10 +4184,14 @@
       <c r="M46" s="45" t="n"/>
       <c r="N46" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O46" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O46" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="45" t="inlineStr">
@@ -4153,10 +4248,14 @@
       <c r="M47" s="45" t="n"/>
       <c r="N47" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O47" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O47" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="45" t="inlineStr">
@@ -4213,10 +4312,14 @@
       <c r="M48" s="45" t="n"/>
       <c r="N48" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O48" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O48" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="45" t="inlineStr">
@@ -4273,10 +4376,14 @@
       <c r="M49" s="45" t="n"/>
       <c r="N49" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O49" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O49" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="45" t="inlineStr">
@@ -4333,10 +4440,14 @@
       <c r="M50" s="45" t="n"/>
       <c r="N50" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O50" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O50" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="45" t="inlineStr">
@@ -4393,10 +4504,14 @@
       <c r="M51" s="45" t="n"/>
       <c r="N51" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O51" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O51" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="45" t="inlineStr">
@@ -4453,10 +4568,14 @@
       <c r="M52" s="45" t="n"/>
       <c r="N52" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O52" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O52" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="45" t="inlineStr">
@@ -4513,10 +4632,14 @@
       <c r="M53" s="45" t="n"/>
       <c r="N53" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O53" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O53" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="45" t="inlineStr">
@@ -4573,10 +4696,14 @@
       <c r="M54" s="45" t="n"/>
       <c r="N54" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O54" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O54" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="45" t="inlineStr">
@@ -4633,10 +4760,14 @@
       <c r="M55" s="45" t="n"/>
       <c r="N55" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O55" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O55" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="45" t="inlineStr">
@@ -4693,10 +4824,14 @@
       <c r="M56" s="45" t="n"/>
       <c r="N56" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O56" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O56" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="45" t="inlineStr">
@@ -4753,10 +4888,14 @@
       <c r="M57" s="45" t="n"/>
       <c r="N57" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O57" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O57" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="45" t="inlineStr">
@@ -4813,10 +4952,14 @@
       <c r="M58" s="45" t="n"/>
       <c r="N58" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O58" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O58" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="45" t="inlineStr">
@@ -4875,10 +5018,14 @@
       <c r="M59" s="45" t="n"/>
       <c r="N59" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O59" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O59" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="45" t="inlineStr">
@@ -4937,10 +5084,14 @@
       <c r="M60" s="45" t="n"/>
       <c r="N60" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O60" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O60" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="45" t="inlineStr">
@@ -4999,10 +5150,14 @@
       <c r="M61" s="45" t="n"/>
       <c r="N61" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O61" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O61" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="45" t="inlineStr">
@@ -5061,10 +5216,14 @@
       <c r="M62" s="45" t="n"/>
       <c r="N62" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O62" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O62" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="45" t="inlineStr">
@@ -5123,10 +5282,14 @@
       <c r="M63" s="45" t="n"/>
       <c r="N63" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O63" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O63" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="45" t="inlineStr">
@@ -5185,10 +5348,14 @@
       <c r="M64" s="45" t="n"/>
       <c r="N64" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O64" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O64" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="45" t="inlineStr">
@@ -5247,10 +5414,14 @@
       <c r="M65" s="45" t="n"/>
       <c r="N65" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O65" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O65" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="45" t="inlineStr">
@@ -5309,10 +5480,14 @@
       <c r="M66" s="45" t="n"/>
       <c r="N66" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O66" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O66" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="45" t="inlineStr">
@@ -5371,10 +5546,14 @@
       <c r="M67" s="45" t="n"/>
       <c r="N67" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O67" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O67" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="45" t="inlineStr">
@@ -5433,10 +5612,14 @@
       <c r="M68" s="45" t="n"/>
       <c r="N68" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O68" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O68" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="45" t="inlineStr">
@@ -5495,10 +5678,14 @@
       <c r="M69" s="45" t="n"/>
       <c r="N69" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O69" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O69" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="B70" s="45" t="inlineStr">
@@ -5557,10 +5744,14 @@
       <c r="M70" s="45" t="n"/>
       <c r="N70" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O70" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O70" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="B71" s="45" t="inlineStr">
@@ -5619,10 +5810,14 @@
       <c r="M71" s="45" t="n"/>
       <c r="N71" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O71" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O71" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="45" t="inlineStr">
@@ -5681,10 +5876,14 @@
       <c r="M72" s="45" t="n"/>
       <c r="N72" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O72" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O72" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="45" t="inlineStr">
@@ -5743,10 +5942,14 @@
       <c r="M73" s="45" t="n"/>
       <c r="N73" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O73" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O73" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="45" t="inlineStr">
@@ -5805,10 +6008,14 @@
       <c r="M74" s="45" t="n"/>
       <c r="N74" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O74" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O74" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="B75" s="45" t="inlineStr">
@@ -5867,10 +6074,14 @@
       <c r="M75" s="45" t="n"/>
       <c r="N75" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O75" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O75" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="B76" s="45" t="inlineStr">
@@ -5929,10 +6140,14 @@
       <c r="M76" s="45" t="n"/>
       <c r="N76" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O76" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O76" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="45" t="inlineStr">
@@ -5991,10 +6206,14 @@
       <c r="M77" s="45" t="n"/>
       <c r="N77" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O77" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O77" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="45" t="inlineStr">
@@ -6053,10 +6272,14 @@
       <c r="M78" s="45" t="n"/>
       <c r="N78" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O78" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O78" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="45" t="inlineStr">
@@ -6115,10 +6338,14 @@
       <c r="M79" s="45" t="n"/>
       <c r="N79" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O79" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O79" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="45" t="inlineStr">
@@ -6177,10 +6404,14 @@
       <c r="M80" s="45" t="n"/>
       <c r="N80" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O80" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O80" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="45" t="inlineStr">
@@ -6239,10 +6470,14 @@
       <c r="M81" s="45" t="n"/>
       <c r="N81" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O81" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O81" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="45" t="inlineStr">
@@ -6301,10 +6536,14 @@
       <c r="M82" s="45" t="n"/>
       <c r="N82" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O82" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O82" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="45" t="inlineStr">
@@ -6363,10 +6602,14 @@
       <c r="M83" s="45" t="n"/>
       <c r="N83" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O83" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O83" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="45" t="inlineStr">
@@ -6425,10 +6668,14 @@
       <c r="M84" s="45" t="n"/>
       <c r="N84" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O84" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O84" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="45" t="inlineStr">
@@ -6487,10 +6734,14 @@
       <c r="M85" s="45" t="n"/>
       <c r="N85" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O85" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O85" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="B86" s="45" t="inlineStr">
@@ -6549,10 +6800,14 @@
       <c r="M86" s="45" t="n"/>
       <c r="N86" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O86" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O86" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="45" t="inlineStr">
@@ -6611,10 +6866,14 @@
       <c r="M87" s="45" t="n"/>
       <c r="N87" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O87" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O87" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="B88" s="45" t="inlineStr">
@@ -6673,10 +6932,14 @@
       <c r="M88" s="45" t="n"/>
       <c r="N88" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O88" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O88" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="45" t="inlineStr">
@@ -6735,10 +6998,14 @@
       <c r="M89" s="45" t="n"/>
       <c r="N89" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O89" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O89" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="B90" s="45" t="inlineStr">
@@ -6797,10 +7064,14 @@
       <c r="M90" s="45" t="n"/>
       <c r="N90" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O90" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O90" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="45" t="inlineStr">
@@ -6859,10 +7130,14 @@
       <c r="M91" s="45" t="n"/>
       <c r="N91" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O91" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O91" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="45" t="inlineStr">
@@ -6921,10 +7196,14 @@
       <c r="M92" s="45" t="n"/>
       <c r="N92" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O92" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O92" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="45" t="inlineStr">
@@ -6983,10 +7262,14 @@
       <c r="M93" s="45" t="n"/>
       <c r="N93" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O93" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O93" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="45" t="inlineStr">
@@ -8363,10 +8646,14 @@
       <c r="M116" s="45" t="n"/>
       <c r="N116" s="45" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O116" s="45" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O116" s="45" t="inlineStr">
+        <is>
+          <t>CHG-UA-2.2-01</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="B117" s="46" t="n"/>

</xml_diff>